<commit_message>
Improve ISSN normalisation and Excel import handling
- Preserve leading zeros when reading XLSX files
- Recover truncated ISSNs including X check digits
- Add ISSN QA reporting and invalid value diagnostics
- Improve handling of malformed source ISSNs
- Add unit tests for ISSN recovery logic
</commit_message>
<xml_diff>
--- a/samples/Cap and Link (CAUL)/CAUL_2025_Cap_Link_SAMPLE_FUN.xlsx
+++ b/samples/Cap and Link (CAUL)/CAUL_2025_Cap_Link_SAMPLE_FUN.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://latrobeuni-my.sharepoint.com/personal/mlawton_ltu_edu_au/Documents/2025/OA Read and Publish/open-access-publishing-and-metrics-pipeline/samples/Cap and Link (CAUL)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://latrobeuni-my.sharepoint.com/personal/mlawton_ltu_edu_au/Documents/Documents/Git/open-access-publishing-metrics-pipeline/samples/Cap and Link (CAUL)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_C27A5ED9F5216A3E0DF90AB6E60A5B3E6112C49F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E63653DD-66ED-4519-BEE5-3B3CD6524A16}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_C27A5ED9F5216A3E0DF90AB6E60A5B3E6112C49F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6404988-D2B1-4EEA-82CD-C6BC617CAD5A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11130" yWindow="12765" windowWidth="21600" windowHeight="15315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Agreement</t>
   </si>
@@ -90,6 +90,15 @@
   </si>
   <si>
     <t>https://airtable.com/shrILLUMINATIstats</t>
+  </si>
+  <si>
+    <t>Journal Type</t>
+  </si>
+  <si>
+    <t>Hybrid</t>
+  </si>
+  <si>
+    <t>Fully Open Access</t>
   </si>
 </sst>
 </file>
@@ -125,45 +134,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -224,6 +204,33 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -238,14 +245,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2520DEF7-37F0-4A02-A0BF-24F07EF1FDE2}" name="Table1" displayName="Table1" ref="A1:E4" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:E4" xr:uid="{2520DEF7-37F0-4A02-A0BF-24F07EF1FDE2}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{03A7FBD5-6349-41E5-ACF4-B5C2068B5DCC}" name="Agreement" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{DAD09774-7301-4F48-86E6-AE5C22DF3D59}" name="Agreement type" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{C6D12C01-AD54-4357-8DA7-92F4A2843D03}" name="Link" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{FD8BA667-B126-482D-A731-7EEE0E194567}" name="Publisher data" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{2F8AC8EA-FB64-4A54-A10B-A73D2732A176}" name="Capped agreement approval statistics" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2520DEF7-37F0-4A02-A0BF-24F07EF1FDE2}" name="Table1" displayName="Table1" ref="A1:F4" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:F4" xr:uid="{2520DEF7-37F0-4A02-A0BF-24F07EF1FDE2}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{03A7FBD5-6349-41E5-ACF4-B5C2068B5DCC}" name="Agreement" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{963B3974-F82E-4CD1-B985-4AB0C4AB354D}" name="Journal Type"/>
+    <tableColumn id="2" xr3:uid="{DAD09774-7301-4F48-86E6-AE5C22DF3D59}" name="Agreement type" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{C6D12C01-AD54-4357-8DA7-92F4A2843D03}" name="Link" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{FD8BA667-B126-482D-A731-7EEE0E194567}" name="Publisher data" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{2F8AC8EA-FB64-4A54-A10B-A73D2732A176}" name="Capped agreement approval statistics" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -538,80 +546,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="36.28515625" customWidth="1"/>
+    <col min="1" max="2" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" customWidth="1"/>
+    <col min="6" max="6" width="36.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>